<commit_message>
add traffic counter with goatcounter
</commit_message>
<xml_diff>
--- a/data/explorer-master.xlsx
+++ b/data/explorer-master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Client Projects\CalCompute\compute-governance-explorer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4048D0-B079-41A4-B921-215163F946D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8CC786-6BDC-4C39-B385-3AAB488E0F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="842" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="842" firstSheet="5" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guide" sheetId="1" r:id="rId1"/>
@@ -4701,9 +4701,6 @@
     <t>footer.license</t>
   </si>
   <si>
-    <t>Code MIT · Data and text CC BY 4.0</t>
-  </si>
-  <si>
     <t>version</t>
   </si>
   <si>
@@ -4792,6 +4789,9 @@
   </si>
   <si>
     <t>Each approach compared by the number of organizations holding layers 2 to 8. Select one to open it in the explorer.</t>
+  </si>
+  <si>
+    <t>Code MIT · Data and text CC BY 4.0; Cookie-free analytics by GoatCounter</t>
   </si>
 </sst>
 </file>
@@ -4799,7 +4799,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -4890,7 +4890,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4908,16 +4908,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5258,7 +5255,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>1559</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="31" x14ac:dyDescent="0.35">
@@ -5308,7 +5305,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>1560</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -5414,7 +5411,7 @@
         <v>38</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>1561</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9330,14 +9327,14 @@
         <v>1488</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>1489</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="11">
         <v>46314</v>
       </c>
     </row>
@@ -9362,7 +9359,7 @@
         <v>1493</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9378,7 +9375,7 @@
         <v>1496</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>1568</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9394,7 +9391,7 @@
         <v>1499</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31" x14ac:dyDescent="0.35">
@@ -9410,7 +9407,7 @@
         <v>1502</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9434,7 +9431,7 @@
         <v>1507</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9450,7 +9447,7 @@
         <v>1510</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>1572</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9458,7 +9455,7 @@
         <v>1511</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>1573</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9498,7 +9495,7 @@
         <v>1520</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>1574</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9506,7 +9503,7 @@
         <v>1521</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>1575</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9530,7 +9527,7 @@
         <v>1526</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9546,7 +9543,7 @@
         <v>1529</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>1577</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9562,7 +9559,7 @@
         <v>1532</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>1578</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9610,7 +9607,7 @@
         <v>1542</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>1579</v>
+        <v>1578</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9626,7 +9623,7 @@
         <v>1544</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9642,7 +9639,7 @@
         <v>1547</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>1564</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -9650,7 +9647,7 @@
         <v>1548</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>1549</v>
+        <v>1579</v>
       </c>
     </row>
   </sheetData>
@@ -9671,57 +9668,57 @@
   <sheetData>
     <row r="1" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
+        <v>1549</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>1550</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>1551</v>
       </c>
-      <c r="C1" s="6" t="s">
-        <v>1552</v>
-      </c>
     </row>
     <row r="2" spans="1:3" s="9" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="4" t="s">
+        <v>1561</v>
+      </c>
+      <c r="B2" s="10">
+        <v>46314</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>1562</v>
-      </c>
-      <c r="B2" s="11">
-        <v>46314</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>1553</v>
+        <v>1552</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>1104</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>1554</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>1555</v>
+        <v>1554</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>1104</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1556</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>1557</v>
+        <v>1556</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>1104</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated changelog with new changes
</commit_message>
<xml_diff>
--- a/data/explorer-master.xlsx
+++ b/data/explorer-master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Client Projects\CalCompute\compute-governance-explorer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8CC786-6BDC-4C39-B385-3AAB488E0F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A08BBE-B196-4EB6-B676-A4B0442E7DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="842" firstSheet="5" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="842" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guide" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Approaches!$A$1:$M$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">Changelog!$A$1:$C$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">Changelog!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Flows!$A$1:$I$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Friction Points'!$A$1:$G$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">Glossary!$A$1:$C$18</definedName>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4667" uniqueCount="1580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4666" uniqueCount="1582">
   <si>
     <t>Compute Stack Explorer: master workbook</t>
   </si>
@@ -4792,6 +4792,12 @@
   </si>
   <si>
     <t>Code MIT · Data and text CC BY 4.0; Cookie-free analytics by GoatCounter</t>
+  </si>
+  <si>
+    <t>1.3.0</t>
+  </si>
+  <si>
+    <t>Added traffic counter and web analytics via goatcounter</t>
   </si>
 </sst>
 </file>
@@ -4890,7 +4896,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4915,6 +4921,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9658,7 +9674,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -9677,52 +9693,63 @@
         <v>1551</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="9" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:3" s="12" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="13" t="s">
+        <v>1580</v>
+      </c>
+      <c r="B2" s="14">
+        <v>46314</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="9" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
         <v>1561</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B3" s="10">
         <v>46314</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>1562</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
         <v>1552</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C3" s="7" t="s">
+      <c r="B4" s="15">
+        <v>46313</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>1553</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="5" spans="1:3" ht="31" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
         <v>1554</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C4" s="7" t="s">
+      <c r="B5" s="15">
+        <v>46313</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>1555</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
         <v>1556</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="B6" s="15">
+        <v>46313</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>1557</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C5" xr:uid="{00000000-0009-0000-0000-000010000000}"/>
+  <autoFilter ref="A1:C6" xr:uid="{00000000-0009-0000-0000-000010000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>